<commit_message>
fix: explain import fields in plain language
</commit_message>
<xml_diff>
--- a/public/templates/竞迹专项训练导入模板.xlsx
+++ b/public/templates/竞迹专项训练导入模板.xlsx
@@ -26,7 +26,7 @@
           <t xml:space="preserve">训练日期
 必填｜YYYY-MM-DD
 例：2026-10-01
-必须填写本次记录的真实日期；不自动补今天。</t>
+必须填写本次记录的真实日期；不自动补今天。 例：2026-10-01</t>
         </r>
       </text>
     </comment>
@@ -34,10 +34,9 @@
       <text>
         <r>
           <t xml:space="preserve">项目
-必填｜无单位
+必填
 例：赛艇
-必须与当前项目空间、所有成员归属一致。
-可选值：赛艇、皮划艇、激流</t>
+必须与当前项目空间、所有成员归属一致。 例：赛艇 可选：赛艇、皮划艇、激流</t>
         </r>
       </text>
     </comment>
@@ -47,7 +46,7 @@
           <t xml:space="preserve">训练距离(m)
 必填｜m
 例：250
-本表用米，不是课次表的千米。</t>
+本表用米，不是课次表的千米。 例：250</t>
         </r>
       </text>
     </comment>
@@ -55,9 +54,9 @@
       <text>
         <r>
           <t xml:space="preserve">艇型
-条件必填｜无单位
+条件必填：需要按艇型、组别排名时填写
 例：按当前项目实际艇型填写
-需要分组排名时必填；留空显示未分组，不与明确分组混排。</t>
+需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：按当前项目实际艇型填写</t>
         </r>
       </text>
     </comment>
@@ -65,9 +64,9 @@
       <text>
         <r>
           <t xml:space="preserve">性别组别
-条件必填｜无单位
+条件必填：需要按艇型、组别排名时填写
 例：男子
-需要分组排名时必填；留空显示未分组，不与明确分组混排。</t>
+需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：男子</t>
         </r>
       </text>
     </comment>
@@ -75,9 +74,9 @@
       <text>
         <r>
           <t xml:space="preserve">运动员/组合
-必填｜无单位
+必填
 例：张某 / 一艇组合
-单人填姓名即可；多人可填写组合名称并在成员列列齐成员。</t>
+单人填姓名即可；多人可填写组合名称并在成员列列齐成员。 例：张某 / 一艇组合</t>
         </r>
       </text>
     </comment>
@@ -85,9 +84,9 @@
       <text>
         <r>
           <t xml:space="preserve">运动员姓名
-条件必填｜无单位
+条件必填：组合名称没有列出完整成员时填写
 例：张某、李某
-组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。</t>
+组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。 例：张某、李某</t>
         </r>
       </text>
     </comment>
@@ -95,9 +94,9 @@
       <text>
         <r>
           <t xml:space="preserve">第1轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:55.15
-至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。</t>
+至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.15</t>
         </r>
       </text>
     </comment>
@@ -105,9 +104,9 @@
       <text>
         <r>
           <t xml:space="preserve">第2轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:56.20
-至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。</t>
+至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:56.20</t>
         </r>
       </text>
     </comment>
@@ -115,9 +114,9 @@
       <text>
         <r>
           <t xml:space="preserve">第3轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:55.80
-至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。</t>
+至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.80</t>
         </r>
       </text>
     </comment>
@@ -125,9 +124,9 @@
       <text>
         <r>
           <t xml:space="preserve">上午/下午
-选填｜无单位
+选填
 例：上午
-仅填写实际已采集数据，未提供留空。</t>
+仅填写实际已采集数据，未提供留空。 例：上午</t>
         </r>
       </text>
     </comment>
@@ -135,9 +134,9 @@
       <text>
         <r>
           <t xml:space="preserve">风向风速
-选填｜无单位
+选填
 例：顺风 1m/s
-仅填写实际已采集数据，未提供留空。</t>
+仅填写实际已采集数据，未提供留空。 例：顺风 1m/s</t>
         </r>
       </text>
     </comment>
@@ -145,9 +144,9 @@
       <text>
         <r>
           <t xml:space="preserve">训练地点
-选填｜无单位
+选填
 例：训练基地
-仅填写实际已采集数据，未提供留空。</t>
+仅填写实际已采集数据，未提供留空。 例：训练基地</t>
         </r>
       </text>
     </comment>
@@ -157,7 +156,7 @@
           <t xml:space="preserve">历史最好
 选填｜m:ss.SS 或秒
 例：0:54.90
-外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。</t>
+外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。 例：0:54.90</t>
         </r>
       </text>
     </comment>
@@ -165,9 +164,9 @@
       <text>
         <r>
           <t xml:space="preserve">备注
-选填｜无单位
+选填
 例：本次实测
-仅填写实际已采集数据，未提供留空。</t>
+仅填写实际已采集数据，未提供留空。 例：本次实测</t>
         </r>
       </text>
     </comment>
@@ -176,7 +175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>竞迹｜专项训练成绩导入模板</t>
   </si>
@@ -208,10 +207,13 @@
     <t>8. 年龄由真实生日计算；冠军模型、雷达图和参考值由系统分析，不要求填报。Excel公式不作为计算事实源。</t>
   </si>
   <si>
-    <t>9. 必填条件见列批注。空白是未提供，真实0保留；非法文本报错。仅预填身份和日期的业务行自动忽略。</t>
-  </si>
-  <si>
-    <t>10. 已有记录只按非空值更新，空白保留已有值；跨项目、越权、同名歧义及同日多课归属必须在提交前解决。</t>
+    <t>9. 表头写明何时填写；点击填写单元格可看解释、填写例子和不知道时的处理办法，详细说明也在表头批注。示例评分表名仅演示格式，请用真实依据，不代表系统提供该标准。</t>
+  </si>
+  <si>
+    <t>10. 必填条件见列批注。空白是未提供，真实0保留；非法文本报错。仅预填身份和日期的业务行自动忽略。</t>
+  </si>
+  <si>
+    <t>11. 已有记录只按非空值更新，空白保留已有值；跨项目、越权、同名歧义及同日多课归属必须在提交前解决。</t>
   </si>
   <si>
     <t>专项训练成绩</t>
@@ -226,7 +228,7 @@
   </si>
   <si>
     <t xml:space="preserve">项目
-必填｜无单位
+必填
 例：赛艇</t>
   </si>
   <si>
@@ -236,52 +238,52 @@
   </si>
   <si>
     <t xml:space="preserve">艇型
-条件必填｜无单位
+条件必填：需要按艇型、组别排名时填写
 例：按当前项目实际艇型填写</t>
   </si>
   <si>
     <t xml:space="preserve">性别组别
-条件必填｜无单位
+条件必填：需要按艇型、组别排名时填写
 例：男子</t>
   </si>
   <si>
     <t xml:space="preserve">运动员/组合
-必填｜无单位
+必填
 例：张某 / 一艇组合</t>
   </si>
   <si>
     <t xml:space="preserve">运动员姓名
-条件必填｜无单位
+条件必填：组合名称没有列出完整成员时填写
 例：张某、李某</t>
   </si>
   <si>
     <t xml:space="preserve">第1轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:55.15</t>
   </si>
   <si>
     <t xml:space="preserve">第2轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:56.20</t>
   </si>
   <si>
     <t xml:space="preserve">第3轮
-条件必填｜m:ss.SS 或秒
+条件必填：三轮至少填一轮，未测轮次留空｜m:ss.SS 或秒
 例：0:55.80</t>
   </si>
   <si>
     <t xml:space="preserve">上午/下午
-选填｜无单位
+选填
 例：上午</t>
   </si>
   <si>
     <t xml:space="preserve">风向风速
-选填｜无单位
+选填
 例：顺风 1m/s</t>
   </si>
   <si>
     <t xml:space="preserve">训练地点
-选填｜无单位
+选填
 例：训练基地</t>
   </si>
   <si>
@@ -291,7 +293,7 @@
   </si>
   <si>
     <t xml:space="preserve">备注
-选填｜无单位
+选填
 例：本次实测</t>
   </si>
 </sst>
@@ -726,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -789,6 +791,11 @@
     <row r="12" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -815,7 +822,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -834,7 +841,7 @@
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -851,51 +858,51 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" ht="82" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" ht="89" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2405,94 +2412,94 @@
     <mergeCell ref="A2:O2"/>
   </mergeCells>
   <dataValidations count="30">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜YYYY-MM-DD" prompt="必须填写本次记录的真实日期；不自动补今天。 例：2026-10-01" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="A10:A503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜YYYY-MM-DD" prompt="必须填写本次记录的真实日期；不自动补今天。 例：2026-10-01" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="A4:A503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="必填｜无单位" prompt="必须与当前项目空间、所有成员归属一致。 例：赛艇" showErrorMessage="1" errorTitle="请检查填写值" error="请选择：赛艇、皮划艇、激流" sqref="B10:B503">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练日期：怎么填" prompt="必须填写本次记录的真实日期；不自动补今天。 例：2026-10-01" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="A10:A503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练日期：怎么填" prompt="必须填写本次记录的真实日期；不自动补今天。 例：2026-10-01" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="A4:A503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="项目：怎么填" prompt="必须与当前项目空间、所有成员归属一致。 例：赛艇 可选：赛艇、皮划艇、激流" showErrorMessage="1" errorTitle="请检查填写值" error="请选择：赛艇、皮划艇、激流" sqref="B10:B503">
       <formula1>"赛艇,皮划艇,激流"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="必填｜无单位" prompt="必须与当前项目空间、所有成员归属一致。 例：赛艇" showErrorMessage="1" errorTitle="请检查填写值" error="请选择：赛艇、皮划艇、激流" sqref="B4:B503">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="项目：怎么填" prompt="必须与当前项目空间、所有成员归属一致。 例：赛艇 可选：赛艇、皮划艇、激流" showErrorMessage="1" errorTitle="请检查填写值" error="请选择：赛艇、皮划艇、激流" sqref="B4:B503">
       <formula1>"赛艇,皮划艇,激流"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜m" prompt="本表用米，不是课次表的千米。 例：250" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="C10:C503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜m" prompt="本表用米，不是课次表的千米。 例：250" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="C4:C503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：按当前项目实际艇型填写" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="D10:D503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：按当前项目实际艇型填写" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="D4:D503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：男子" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="E10:E503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：男子" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="E4:E503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜无单位" prompt="单人填姓名即可；多人可填写组合名称并在成员列列齐成员。 例：张某 / 一艇组合" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="F10:F503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="必填｜无单位" prompt="单人填姓名即可；多人可填写组合名称并在成员列列齐成员。 例：张某 / 一艇组合" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="F4:F503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。 例：张某、李某" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="G10:G503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜无单位" prompt="组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。 例：张某、李某" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="G4:G503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.15" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="H10:H503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.15" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="H4:H503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:56.20" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="I10:I503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:56.20" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="I4:I503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.80" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="J10:J503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="条件必填｜m:ss.SS 或秒" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.80" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="J4:J503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：上午" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="K10:K503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：上午" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="K4:K503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：顺风 1m/s" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="L10:L503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：顺风 1m/s" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="L4:L503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：训练基地" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="M10:M503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：训练基地" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="M4:M503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜m:ss.SS 或秒" prompt="外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。 例：0:54.90" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="N10:N503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜m:ss.SS 或秒" prompt="外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。 例：0:54.90" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="N4:N503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：本次实测" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="O10:O503">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="选填｜无单位" prompt="仅填写实际已采集数据，未提供留空。 例：本次实测" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="O4:O503">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练距离(m)：怎么填" prompt="本表用米，不是课次表的千米。 例：250" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="C10:C503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练距离(m)：怎么填" prompt="本表用米，不是课次表的千米。 例：250" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="C4:C503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="艇型：怎么填" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：按当前项目实际艇型填写" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="D10:D503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="艇型：怎么填" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：按当前项目实际艇型填写" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="D4:D503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="性别组别：怎么填" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：男子" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="E10:E503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="性别组别：怎么填" prompt="需要分组排名时必填；留空显示未分组，不与明确分组混排。 例：男子" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="E4:E503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="运动员/组合：怎么填" prompt="单人填姓名即可；多人可填写组合名称并在成员列列齐成员。 例：张某 / 一艇组合" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="F10:F503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="运动员/组合：怎么填" prompt="单人填姓名即可；多人可填写组合名称并在成员列列齐成员。 例：张某 / 一艇组合" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="F4:F503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="运动员姓名：怎么填" prompt="组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。 例：张某、李某" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="G10:G503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="运动员姓名：怎么填" prompt="组合名称未列出完整成员时必填，成员用“、”分隔；单人无需重复填姓名。 例：张某、李某" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="G4:G503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第1轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.15" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="H10:H503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第1轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.15" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="H4:H503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第2轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:56.20" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="I10:I503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第2轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:56.20" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="I4:I503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第3轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.80" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="J10:J503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="第3轮：怎么填" prompt="至少一轮有效成绩；第2、3轮未测留空，系统计算有效轮次平均和最好成绩。 例：0:55.80" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="J4:J503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="上午/下午：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：上午" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="K10:K503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="上午/下午：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：上午" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="K4:K503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="风向风速：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：顺风 1m/s" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="L10:L503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="风向风速：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：顺风 1m/s" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="L4:L503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练地点：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：训练基地" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="M10:M503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="训练地点：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：训练基地" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="M4:M503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="历史最好：怎么填" prompt="外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。 例：0:54.90" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="N10:N503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="历史最好：怎么填" prompt="外部已知历史原值选填；不要求手算，比较必须满足既有可比条件。 例：0:54.90" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="N4:N503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="备注：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：本次实测" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="O10:O503">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="备注：怎么填" prompt="仅填写实际已采集数据，未提供留空。 例：本次实测" errorTitle="请检查填写值" error="请选择：按列说明填写" sqref="O4:O503">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: show optional import columns after required fields
</commit_message>
<xml_diff>
--- a/public/templates/竞迹专项训练导入模板.xlsx
+++ b/public/templates/竞迹专项训练导入模板.xlsx
@@ -183,10 +183,10 @@
     <t>jingji-import-v2</t>
   </si>
   <si>
-    <t>1. 常用列在前；专业选填列在右侧默认收起，点左上角分组级别“2”展开。不支持分组时使用取消隐藏列；不使用宏。</t>
-  </si>
-  <si>
-    <t>2. 第1—3行是说明和表头，第4行起填写；示例仅在表头，不需要删除示例数据。隐藏列有值仍会校验和导入。</t>
+    <t>1. 必填项在前，选填项在后；常用选填项排在专业选填项前面，所有数据列直接显示，按需填写即可。</t>
+  </si>
+  <si>
+    <t>2. 第1—3行是说明和表头，第4行起填写；示例仅在表头，不需要删除示例数据。所有已填写的数据都会校验和导入。</t>
   </si>
   <si>
     <t>3. 业务日期须在行内填写，或在上传页明确选择统一日期；新模板不静默使用今天，生日永不补填。</t>
@@ -219,7 +219,7 @@
     <t>专项训练成绩</t>
   </si>
   <si>
-    <t>每个运动员或组合的一次专项成绩一行；日期、项目、距离(m)、运动员/组合、至少一轮成绩必需。单人只填一次姓名；组合需完整成员；艇型/组别缺省为未分组，不与明确分组混排。 专业选填列已收起，点左上角分组级别“2”展开；不支持分组时取消隐藏列。详情见列批注。</t>
+    <t>每个运动员或组合的一次专项成绩一行；日期、项目、距离(m)、运动员/组合、至少一轮成绩必需。单人只填一次姓名；组合需完整成员；艇型/组别缺省为未分组，不与明确分组混排。 必填项在前，选填项在后；所有数据列直接显示，按需填写。详情见列批注。</t>
   </si>
   <si>
     <t xml:space="preserve">训练日期
@@ -806,18 +806,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
   <dimension ref="A1:O503"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="1" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" style="3" customWidth="1"/>
     <col min="2" max="5" width="22" customWidth="1"/>
     <col min="6" max="7" width="28" customWidth="1"/>
-    <col min="8" max="11" width="22" customWidth="1"/>
-    <col min="12" max="14" width="22" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
-    <col min="15" max="15" width="28" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="8" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
style: distinguish import requirements with contrasting colors
</commit_message>
<xml_diff>
--- a/public/templates/竞迹专项训练导入模板.xlsx
+++ b/public/templates/竞迹专项训练导入模板.xlsx
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>竞迹｜专项训练成绩导入模板</t>
   </si>
@@ -183,37 +183,40 @@
     <t>jingji-import-v2</t>
   </si>
   <si>
-    <t>1. 必填项在前，选填项在后；常用选填项排在专业选填项前面，所有数据列直接显示，按需填写即可。</t>
-  </si>
-  <si>
-    <t>2. 第1—3行是说明和表头，第4行起填写；示例仅在表头，不需要删除示例数据。所有已填写的数据都会校验和导入。</t>
-  </si>
-  <si>
-    <t>3. 业务日期须在行内填写，或在上传页明确选择统一日期；新模板不静默使用今天，生日永不补填。</t>
-  </si>
-  <si>
-    <t>4. 系统预填：授权范围内的人员编号、姓名、项目和队伍；不要自行编造编号，不预填测量成绩。</t>
-  </si>
-  <si>
-    <t>5. SRPE：有效时长(min)×RPE，单位AU；缺时长或RPE保持未提供，不能根据距离推算时长。</t>
-  </si>
-  <si>
-    <t>6. SMVL/力量训练量：按现有规则汇总实际次数×实际重量kg；计划数不是实际数，外部显式总量沿用既有优先策略。</t>
-  </si>
-  <si>
-    <t>7. FMS：七项齐全才生成完整21分制总分，未测不补0。专项：按有效轮次计算平均、最好及同条件排名；无可比历史显示缺失。</t>
-  </si>
-  <si>
-    <t>8. 年龄由真实生日计算；冠军模型、雷达图和参考值由系统分析，不要求填报。Excel公式不作为计算事实源。</t>
-  </si>
-  <si>
-    <t>9. 表头写明何时填写；点击填写单元格可看解释、填写例子和不知道时的处理办法，详细说明也在表头批注。示例评分表名仅演示格式，请用真实依据，不代表系统提供该标准。</t>
-  </si>
-  <si>
-    <t>10. 必填条件见列批注。空白是未提供，真实0保留；非法文本报错。仅预填身份和日期的业务行自动忽略。</t>
-  </si>
-  <si>
-    <t>11. 已有记录只按非空值更新，空白保留已有值；跨项目、越权、同名歧义及同日多课归属必须在提交前解决。</t>
+    <t>1. 表头颜色：红色=必填，橙色=满足说明中的条件才必填，蓝色=选填，灰色=系统预填；具体填写要求以表头文字为准。</t>
+  </si>
+  <si>
+    <t>2. 必填项在前，选填项在后；常用选填项排在专业选填项前面，所有数据列直接显示，按需填写即可。</t>
+  </si>
+  <si>
+    <t>3. 第1—3行是说明和表头，第4行起填写；示例仅在表头，不需要删除示例数据。所有已填写的数据都会校验和导入。</t>
+  </si>
+  <si>
+    <t>4. 业务日期须在行内填写，或在上传页明确选择统一日期；新模板不静默使用今天，生日永不补填。</t>
+  </si>
+  <si>
+    <t>5. 系统预填：授权范围内的人员编号、姓名、项目和队伍；不要自行编造编号，不预填测量成绩。</t>
+  </si>
+  <si>
+    <t>6. SRPE：有效时长(min)×RPE，单位AU；缺时长或RPE保持未提供，不能根据距离推算时长。</t>
+  </si>
+  <si>
+    <t>7. SMVL/力量训练量：按现有规则汇总实际次数×实际重量kg；计划数不是实际数，外部显式总量沿用既有优先策略。</t>
+  </si>
+  <si>
+    <t>8. FMS：七项齐全才生成完整21分制总分，未测不补0。专项：按有效轮次计算平均、最好及同条件排名；无可比历史显示缺失。</t>
+  </si>
+  <si>
+    <t>9. 年龄由真实生日计算；冠军模型、雷达图和参考值由系统分析，不要求填报。Excel公式不作为计算事实源。</t>
+  </si>
+  <si>
+    <t>10. 表头写明何时填写；点击填写单元格可看解释、填写例子和不知道时的处理办法，详细说明也在表头批注。示例评分表名仅演示格式，请用真实依据，不代表系统提供该标准。</t>
+  </si>
+  <si>
+    <t>11. 必填条件见列批注。空白是未提供，真实0保留；非法文本报错。仅预填身份和日期的业务行自动忽略。</t>
+  </si>
+  <si>
+    <t>12. 已有记录只按非空值更新，空白保留已有值；跨项目、越权、同名歧义及同日多课归属必须在提交前解决。</t>
   </si>
   <si>
     <t>专项训练成绩</t>
@@ -304,7 +307,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -325,6 +328,10 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF422006"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -340,17 +347,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF193A44"/>
+        <fgColor rgb="FF991B1B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF345D68"/>
+        <fgColor rgb="FFF59E0B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF52747C"/>
+        <fgColor rgb="FF1D4ED8"/>
       </patternFill>
     </fill>
   </fills>
@@ -383,7 +390,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -728,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -796,6 +803,11 @@
     <row r="13" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -818,7 +830,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -837,7 +849,7 @@
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -856,49 +868,49 @@
     </row>
     <row r="3" ht="89" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>